<commit_message>
Update Tentative Schedule (Spring 2026).xlsx
</commit_message>
<xml_diff>
--- a/Intro materials/Tentative Schedule (Spring 2026).xlsx
+++ b/Intro materials/Tentative Schedule (Spring 2026).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamsoliman/Documents/GitHub/Econometrics-Slides/Intro materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C65F02BA-34D4-0745-A1E4-201D941EA74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8556A933-774B-ED41-9C1B-E329119E11C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15180" xr2:uid="{72D0DB20-A265-EC45-9D54-DA8133B16545}"/>
   </bookViews>
@@ -714,21 +714,21 @@
       </c>
     </row>
     <row r="25" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="6">
+      <c r="A25" s="7">
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="6">
+        <f t="shared" si="0"/>
+        <v>46114</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="7">
-        <f t="shared" si="0"/>
-        <v>46114</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>